<commit_message>
Intégration du backend ML, tests et correction de bugs
</commit_message>
<xml_diff>
--- a/data/raw/ccn_cybersec.xlsx
+++ b/data/raw/ccn_cybersec.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1ère Année" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2ème Année" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3ème Année" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -113,8 +114,63 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00888888"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007030A0"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="40">
     <fill>
       <patternFill/>
     </fill>
@@ -242,8 +298,93 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D6A9F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF9900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0E4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE1F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FFFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FFFD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -313,6 +454,50 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -324,7 +509,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -479,6 +664,78 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="19" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="26" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="30" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="31" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="27" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="36" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="34" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="38" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="39" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4037,7 +4294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Z39"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="22" min="1" max="1"/>
@@ -7321,6 +7578,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="N2:W2"/>
@@ -7333,4 +7591,1125 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="23" min="1" max="1"/>
+    <col width="16" customWidth="1" style="23" min="2" max="2"/>
+    <col width="14" customWidth="1" style="23" min="3" max="3"/>
+    <col width="11" customWidth="1" style="23" min="4" max="4"/>
+    <col width="22" customWidth="1" style="23" min="5" max="5"/>
+    <col width="22" customWidth="1" style="23" min="6" max="6"/>
+    <col width="22" customWidth="1" style="23" min="7" max="7"/>
+    <col width="22" customWidth="1" style="23" min="8" max="8"/>
+    <col width="22" customWidth="1" style="23" min="9" max="9"/>
+    <col width="22" customWidth="1" style="23" min="10" max="10"/>
+    <col width="22" customWidth="1" style="23" min="11" max="11"/>
+    <col width="3" customWidth="1" style="23" min="12" max="12"/>
+    <col width="13" customWidth="1" style="23" min="13" max="13"/>
+    <col width="14" customWidth="1" style="23" min="14" max="14"/>
+    <col width="15" customWidth="1" style="23" min="15" max="15"/>
+    <col width="12" customWidth="1" style="23" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" s="23">
+      <c r="A1" s="53" t="inlineStr">
+        <is>
+          <t>DÉPARTEMENT CCN CYBERSÉCURITÉ — TROISIÈME ANNÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="23">
+      <c r="A2" s="54" t="inlineStr">
+        <is>
+          <t>Informations Générales</t>
+        </is>
+      </c>
+      <c r="D2" s="54" t="inlineStr">
+        <is>
+          <t>SEMESTRE 5</t>
+        </is>
+      </c>
+      <c r="N2" s="54" t="inlineStr">
+        <is>
+          <t>SEMESTRE 6</t>
+        </is>
+      </c>
+      <c r="O2" s="54" t="n"/>
+      <c r="P2" s="54" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="23">
+      <c r="A3" s="55" t="n"/>
+      <c r="D3" s="56" t="n"/>
+      <c r="E3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 5</t>
+        </is>
+      </c>
+      <c r="F3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 5</t>
+        </is>
+      </c>
+      <c r="G3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 5</t>
+        </is>
+      </c>
+      <c r="H3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 4</t>
+        </is>
+      </c>
+      <c r="I3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 4</t>
+        </is>
+      </c>
+      <c r="J3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 3</t>
+        </is>
+      </c>
+      <c r="K3" s="56" t="inlineStr">
+        <is>
+          <t>Coef 3</t>
+        </is>
+      </c>
+      <c r="M3" s="56" t="n"/>
+      <c r="N3" s="70" t="inlineStr">
+        <is>
+          <t>Coef 20</t>
+        </is>
+      </c>
+      <c r="O3" s="56" t="n"/>
+      <c r="P3" s="56" t="n"/>
+    </row>
+    <row r="4" ht="54" customHeight="1" s="23">
+      <c r="A4" s="57" t="inlineStr">
+        <is>
+          <t>CNE</t>
+        </is>
+      </c>
+      <c r="B4" s="57" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="C4" s="57" t="inlineStr">
+        <is>
+          <t>Prénom</t>
+        </is>
+      </c>
+      <c r="D4" s="54" t="inlineStr">
+        <is>
+          <t>Absences S5</t>
+        </is>
+      </c>
+      <c r="E4" s="58" t="inlineStr">
+        <is>
+          <t>Cryptographie Post-Quantique</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
+        <is>
+          <t>SOC et SIEM</t>
+        </is>
+      </c>
+      <c r="G4" s="58" t="inlineStr">
+        <is>
+          <t>Mathématiques 5</t>
+        </is>
+      </c>
+      <c r="H4" s="58" t="inlineStr">
+        <is>
+          <t>Pentest Avancé</t>
+        </is>
+      </c>
+      <c r="I4" s="58" t="inlineStr">
+        <is>
+          <t>Sécurité des Systèmes Industriels</t>
+        </is>
+      </c>
+      <c r="J4" s="58" t="inlineStr">
+        <is>
+          <t>Anglais Professionnel</t>
+        </is>
+      </c>
+      <c r="K4" s="58" t="inlineStr">
+        <is>
+          <t>Français Professionnel 5</t>
+        </is>
+      </c>
+      <c r="M4" s="59" t="inlineStr">
+        <is>
+          <t>Moyenne
+SEMESTRE 5</t>
+        </is>
+      </c>
+      <c r="N4" s="71" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="O4" s="62" t="inlineStr">
+        <is>
+          <t>Moyenne
+Annuelle
+3ème Année</t>
+        </is>
+      </c>
+      <c r="P4" s="63" t="inlineStr">
+        <is>
+          <t>Redoublant</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="23">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>B441737</t>
+        </is>
+      </c>
+      <c r="B5" s="64" t="inlineStr">
+        <is>
+          <t>Bensouda</t>
+        </is>
+      </c>
+      <c r="C5" s="64" t="inlineStr">
+        <is>
+          <t>Khalil</t>
+        </is>
+      </c>
+      <c r="D5" s="72" t="n"/>
+      <c r="E5" s="66" t="n"/>
+      <c r="F5" s="66" t="n"/>
+      <c r="G5" s="66" t="n"/>
+      <c r="H5" s="66" t="n"/>
+      <c r="I5" s="66" t="n"/>
+      <c r="J5" s="66" t="n"/>
+      <c r="K5" s="66" t="n"/>
+      <c r="L5" s="73" t="n"/>
+      <c r="M5" s="48" t="n"/>
+      <c r="N5" s="74" t="n"/>
+      <c r="O5" s="75" t="n"/>
+      <c r="P5" s="68" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="23">
+      <c r="A6" s="76" t="inlineStr">
+        <is>
+          <t>R352175</t>
+        </is>
+      </c>
+      <c r="B6" s="76" t="inlineStr">
+        <is>
+          <t>Chraibi</t>
+        </is>
+      </c>
+      <c r="C6" s="76" t="inlineStr">
+        <is>
+          <t>Nora</t>
+        </is>
+      </c>
+      <c r="D6" s="72" t="n"/>
+      <c r="E6" s="66" t="n"/>
+      <c r="F6" s="66" t="n"/>
+      <c r="G6" s="66" t="n"/>
+      <c r="H6" s="66" t="n"/>
+      <c r="I6" s="66" t="n"/>
+      <c r="J6" s="66" t="n"/>
+      <c r="K6" s="66" t="n"/>
+      <c r="L6" s="73" t="n"/>
+      <c r="M6" s="48" t="n"/>
+      <c r="N6" s="74" t="n"/>
+      <c r="O6" s="75" t="n"/>
+      <c r="P6" s="68" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="23">
+      <c r="A7" s="64" t="inlineStr">
+        <is>
+          <t>R962512</t>
+        </is>
+      </c>
+      <c r="B7" s="64" t="inlineStr">
+        <is>
+          <t>Daoudi</t>
+        </is>
+      </c>
+      <c r="C7" s="64" t="inlineStr">
+        <is>
+          <t>Yassine</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="n"/>
+      <c r="E7" s="66" t="n"/>
+      <c r="F7" s="66" t="n"/>
+      <c r="G7" s="66" t="n"/>
+      <c r="H7" s="66" t="n"/>
+      <c r="I7" s="66" t="n"/>
+      <c r="J7" s="66" t="n"/>
+      <c r="K7" s="66" t="n"/>
+      <c r="L7" s="73" t="n"/>
+      <c r="M7" s="48" t="n"/>
+      <c r="N7" s="74" t="n"/>
+      <c r="O7" s="75" t="n"/>
+      <c r="P7" s="68" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="23">
+      <c r="A8" s="76" t="inlineStr">
+        <is>
+          <t>F406524</t>
+        </is>
+      </c>
+      <c r="B8" s="76" t="inlineStr">
+        <is>
+          <t>Ennaji</t>
+        </is>
+      </c>
+      <c r="C8" s="76" t="inlineStr">
+        <is>
+          <t>Samira</t>
+        </is>
+      </c>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="66" t="n"/>
+      <c r="F8" s="66" t="n"/>
+      <c r="G8" s="66" t="n"/>
+      <c r="H8" s="66" t="n"/>
+      <c r="I8" s="66" t="n"/>
+      <c r="J8" s="66" t="n"/>
+      <c r="K8" s="66" t="n"/>
+      <c r="L8" s="73" t="n"/>
+      <c r="M8" s="48" t="n"/>
+      <c r="N8" s="74" t="n"/>
+      <c r="O8" s="75" t="n"/>
+      <c r="P8" s="68" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="23">
+      <c r="A9" s="64" t="inlineStr">
+        <is>
+          <t>G684995</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="inlineStr">
+        <is>
+          <t>Fadili</t>
+        </is>
+      </c>
+      <c r="C9" s="64" t="inlineStr">
+        <is>
+          <t>Hamza</t>
+        </is>
+      </c>
+      <c r="D9" s="72" t="n"/>
+      <c r="E9" s="66" t="n"/>
+      <c r="F9" s="66" t="n"/>
+      <c r="G9" s="66" t="n"/>
+      <c r="H9" s="66" t="n"/>
+      <c r="I9" s="66" t="n"/>
+      <c r="J9" s="66" t="n"/>
+      <c r="K9" s="66" t="n"/>
+      <c r="L9" s="73" t="n"/>
+      <c r="M9" s="48" t="n"/>
+      <c r="N9" s="74" t="n"/>
+      <c r="O9" s="75" t="n"/>
+      <c r="P9" s="68" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="23">
+      <c r="A10" s="76" t="inlineStr">
+        <is>
+          <t>P349362</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>Ghriss</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>Imane</t>
+        </is>
+      </c>
+      <c r="D10" s="72" t="n"/>
+      <c r="E10" s="66" t="n"/>
+      <c r="F10" s="66" t="n"/>
+      <c r="G10" s="66" t="n"/>
+      <c r="H10" s="66" t="n"/>
+      <c r="I10" s="66" t="n"/>
+      <c r="J10" s="66" t="n"/>
+      <c r="K10" s="66" t="n"/>
+      <c r="L10" s="73" t="n"/>
+      <c r="M10" s="48" t="n"/>
+      <c r="N10" s="74" t="n"/>
+      <c r="O10" s="75" t="n"/>
+      <c r="P10" s="68" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="23">
+      <c r="A11" s="64" t="inlineStr">
+        <is>
+          <t>H682893</t>
+        </is>
+      </c>
+      <c r="B11" s="64" t="inlineStr">
+        <is>
+          <t>Hajjioui</t>
+        </is>
+      </c>
+      <c r="C11" s="64" t="inlineStr">
+        <is>
+          <t>Tarik</t>
+        </is>
+      </c>
+      <c r="D11" s="72" t="n"/>
+      <c r="E11" s="66" t="n"/>
+      <c r="F11" s="66" t="n"/>
+      <c r="G11" s="66" t="n"/>
+      <c r="H11" s="66" t="n"/>
+      <c r="I11" s="66" t="n"/>
+      <c r="J11" s="66" t="n"/>
+      <c r="K11" s="66" t="n"/>
+      <c r="L11" s="73" t="n"/>
+      <c r="M11" s="48" t="n"/>
+      <c r="N11" s="74" t="n"/>
+      <c r="O11" s="75" t="n"/>
+      <c r="P11" s="68" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="23">
+      <c r="A12" s="76" t="inlineStr">
+        <is>
+          <t>N102544</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>Idrissi</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>Rania</t>
+        </is>
+      </c>
+      <c r="D12" s="72" t="n"/>
+      <c r="E12" s="66" t="n"/>
+      <c r="F12" s="66" t="n"/>
+      <c r="G12" s="66" t="n"/>
+      <c r="H12" s="66" t="n"/>
+      <c r="I12" s="66" t="n"/>
+      <c r="J12" s="66" t="n"/>
+      <c r="K12" s="66" t="n"/>
+      <c r="L12" s="73" t="n"/>
+      <c r="M12" s="48" t="n"/>
+      <c r="N12" s="74" t="n"/>
+      <c r="O12" s="75" t="n"/>
+      <c r="P12" s="68" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="23">
+      <c r="A13" s="64" t="inlineStr">
+        <is>
+          <t>B129728</t>
+        </is>
+      </c>
+      <c r="B13" s="64" t="inlineStr">
+        <is>
+          <t>Jebli</t>
+        </is>
+      </c>
+      <c r="C13" s="64" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
+        </is>
+      </c>
+      <c r="D13" s="72" t="n"/>
+      <c r="E13" s="66" t="n"/>
+      <c r="F13" s="66" t="n"/>
+      <c r="G13" s="66" t="n"/>
+      <c r="H13" s="66" t="n"/>
+      <c r="I13" s="66" t="n"/>
+      <c r="J13" s="66" t="n"/>
+      <c r="K13" s="66" t="n"/>
+      <c r="L13" s="73" t="n"/>
+      <c r="M13" s="48" t="n"/>
+      <c r="N13" s="74" t="n"/>
+      <c r="O13" s="75" t="n"/>
+      <c r="P13" s="68" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="23">
+      <c r="A14" s="76" t="inlineStr">
+        <is>
+          <t>G281067</t>
+        </is>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>Karoumi</t>
+        </is>
+      </c>
+      <c r="C14" s="76" t="inlineStr">
+        <is>
+          <t>Dounia</t>
+        </is>
+      </c>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="66" t="n"/>
+      <c r="F14" s="66" t="n"/>
+      <c r="G14" s="66" t="n"/>
+      <c r="H14" s="66" t="n"/>
+      <c r="I14" s="66" t="n"/>
+      <c r="J14" s="66" t="n"/>
+      <c r="K14" s="66" t="n"/>
+      <c r="L14" s="73" t="n"/>
+      <c r="M14" s="48" t="n"/>
+      <c r="N14" s="74" t="n"/>
+      <c r="O14" s="75" t="n"/>
+      <c r="P14" s="68" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="23">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>R631958</t>
+        </is>
+      </c>
+      <c r="B15" s="64" t="inlineStr">
+        <is>
+          <t>Lahlali</t>
+        </is>
+      </c>
+      <c r="C15" s="64" t="inlineStr">
+        <is>
+          <t>Anas</t>
+        </is>
+      </c>
+      <c r="D15" s="72" t="n"/>
+      <c r="E15" s="66" t="n"/>
+      <c r="F15" s="66" t="n"/>
+      <c r="G15" s="66" t="n"/>
+      <c r="H15" s="66" t="n"/>
+      <c r="I15" s="66" t="n"/>
+      <c r="J15" s="66" t="n"/>
+      <c r="K15" s="66" t="n"/>
+      <c r="L15" s="73" t="n"/>
+      <c r="M15" s="48" t="n"/>
+      <c r="N15" s="74" t="n"/>
+      <c r="O15" s="75" t="n"/>
+      <c r="P15" s="68" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="23">
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>M291757</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>Moutaouakil</t>
+        </is>
+      </c>
+      <c r="C16" s="76" t="inlineStr">
+        <is>
+          <t>Sara</t>
+        </is>
+      </c>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="66" t="n"/>
+      <c r="F16" s="66" t="n"/>
+      <c r="G16" s="66" t="n"/>
+      <c r="H16" s="66" t="n"/>
+      <c r="I16" s="66" t="n"/>
+      <c r="J16" s="66" t="n"/>
+      <c r="K16" s="66" t="n"/>
+      <c r="L16" s="73" t="n"/>
+      <c r="M16" s="48" t="n"/>
+      <c r="N16" s="74" t="n"/>
+      <c r="O16" s="75" t="n"/>
+      <c r="P16" s="68" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="23">
+      <c r="A17" s="64" t="inlineStr">
+        <is>
+          <t>T437098</t>
+        </is>
+      </c>
+      <c r="B17" s="64" t="inlineStr">
+        <is>
+          <t>Nouri</t>
+        </is>
+      </c>
+      <c r="C17" s="64" t="inlineStr">
+        <is>
+          <t>Bilal</t>
+        </is>
+      </c>
+      <c r="D17" s="72" t="n"/>
+      <c r="E17" s="66" t="n"/>
+      <c r="F17" s="66" t="n"/>
+      <c r="G17" s="66" t="n"/>
+      <c r="H17" s="66" t="n"/>
+      <c r="I17" s="66" t="n"/>
+      <c r="J17" s="66" t="n"/>
+      <c r="K17" s="66" t="n"/>
+      <c r="L17" s="73" t="n"/>
+      <c r="M17" s="48" t="n"/>
+      <c r="N17" s="74" t="n"/>
+      <c r="O17" s="75" t="n"/>
+      <c r="P17" s="68" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="23">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>F191417</t>
+        </is>
+      </c>
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t>Ouazzani</t>
+        </is>
+      </c>
+      <c r="C18" s="76" t="inlineStr">
+        <is>
+          <t>Fatima</t>
+        </is>
+      </c>
+      <c r="D18" s="72" t="n"/>
+      <c r="E18" s="66" t="n"/>
+      <c r="F18" s="66" t="n"/>
+      <c r="G18" s="66" t="n"/>
+      <c r="H18" s="66" t="n"/>
+      <c r="I18" s="66" t="n"/>
+      <c r="J18" s="66" t="n"/>
+      <c r="K18" s="66" t="n"/>
+      <c r="L18" s="73" t="n"/>
+      <c r="M18" s="48" t="n"/>
+      <c r="N18" s="74" t="n"/>
+      <c r="O18" s="75" t="n"/>
+      <c r="P18" s="68" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="23">
+      <c r="A19" s="64" t="inlineStr">
+        <is>
+          <t>N916546</t>
+        </is>
+      </c>
+      <c r="B19" s="64" t="inlineStr">
+        <is>
+          <t>Patel</t>
+        </is>
+      </c>
+      <c r="C19" s="64" t="inlineStr">
+        <is>
+          <t>Karim</t>
+        </is>
+      </c>
+      <c r="D19" s="72" t="n"/>
+      <c r="E19" s="66" t="n"/>
+      <c r="F19" s="66" t="n"/>
+      <c r="G19" s="66" t="n"/>
+      <c r="H19" s="66" t="n"/>
+      <c r="I19" s="66" t="n"/>
+      <c r="J19" s="66" t="n"/>
+      <c r="K19" s="66" t="n"/>
+      <c r="L19" s="73" t="n"/>
+      <c r="M19" s="48" t="n"/>
+      <c r="N19" s="74" t="n"/>
+      <c r="O19" s="75" t="n"/>
+      <c r="P19" s="68" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="23">
+      <c r="A20" s="76" t="inlineStr">
+        <is>
+          <t>B659906</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>Qorchi</t>
+        </is>
+      </c>
+      <c r="C20" s="76" t="inlineStr">
+        <is>
+          <t>Houda</t>
+        </is>
+      </c>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="66" t="n"/>
+      <c r="F20" s="66" t="n"/>
+      <c r="G20" s="66" t="n"/>
+      <c r="H20" s="66" t="n"/>
+      <c r="I20" s="66" t="n"/>
+      <c r="J20" s="66" t="n"/>
+      <c r="K20" s="66" t="n"/>
+      <c r="L20" s="73" t="n"/>
+      <c r="M20" s="48" t="n"/>
+      <c r="N20" s="74" t="n"/>
+      <c r="O20" s="75" t="n"/>
+      <c r="P20" s="68" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="23">
+      <c r="A21" s="64" t="inlineStr">
+        <is>
+          <t>G314933</t>
+        </is>
+      </c>
+      <c r="B21" s="64" t="inlineStr">
+        <is>
+          <t>Rahali</t>
+        </is>
+      </c>
+      <c r="C21" s="64" t="inlineStr">
+        <is>
+          <t>Zakaria</t>
+        </is>
+      </c>
+      <c r="D21" s="72" t="n"/>
+      <c r="E21" s="66" t="n"/>
+      <c r="F21" s="66" t="n"/>
+      <c r="G21" s="66" t="n"/>
+      <c r="H21" s="66" t="n"/>
+      <c r="I21" s="66" t="n"/>
+      <c r="J21" s="66" t="n"/>
+      <c r="K21" s="66" t="n"/>
+      <c r="L21" s="73" t="n"/>
+      <c r="M21" s="48" t="n"/>
+      <c r="N21" s="74" t="n"/>
+      <c r="O21" s="75" t="n"/>
+      <c r="P21" s="68" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="23">
+      <c r="A22" s="76" t="inlineStr">
+        <is>
+          <t>R300999</t>
+        </is>
+      </c>
+      <c r="B22" s="76" t="inlineStr">
+        <is>
+          <t>Sabbar</t>
+        </is>
+      </c>
+      <c r="C22" s="76" t="inlineStr">
+        <is>
+          <t>Meriem</t>
+        </is>
+      </c>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="66" t="n"/>
+      <c r="F22" s="66" t="n"/>
+      <c r="G22" s="66" t="n"/>
+      <c r="H22" s="66" t="n"/>
+      <c r="I22" s="66" t="n"/>
+      <c r="J22" s="66" t="n"/>
+      <c r="K22" s="66" t="n"/>
+      <c r="L22" s="73" t="n"/>
+      <c r="M22" s="48" t="n"/>
+      <c r="N22" s="74" t="n"/>
+      <c r="O22" s="75" t="n"/>
+      <c r="P22" s="68" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="23">
+      <c r="A23" s="64" t="inlineStr">
+        <is>
+          <t>F184881</t>
+        </is>
+      </c>
+      <c r="B23" s="64" t="inlineStr">
+        <is>
+          <t>Tahiri</t>
+        </is>
+      </c>
+      <c r="C23" s="64" t="inlineStr">
+        <is>
+          <t>Othmane</t>
+        </is>
+      </c>
+      <c r="D23" s="72" t="n"/>
+      <c r="E23" s="66" t="n"/>
+      <c r="F23" s="66" t="n"/>
+      <c r="G23" s="66" t="n"/>
+      <c r="H23" s="66" t="n"/>
+      <c r="I23" s="66" t="n"/>
+      <c r="J23" s="66" t="n"/>
+      <c r="K23" s="66" t="n"/>
+      <c r="L23" s="73" t="n"/>
+      <c r="M23" s="48" t="n"/>
+      <c r="N23" s="74" t="n"/>
+      <c r="O23" s="75" t="n"/>
+      <c r="P23" s="68" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="23">
+      <c r="A24" s="76" t="inlineStr">
+        <is>
+          <t>R831099</t>
+        </is>
+      </c>
+      <c r="B24" s="76" t="inlineStr">
+        <is>
+          <t>Ujjain</t>
+        </is>
+      </c>
+      <c r="C24" s="76" t="inlineStr">
+        <is>
+          <t>Widad</t>
+        </is>
+      </c>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="66" t="n"/>
+      <c r="F24" s="66" t="n"/>
+      <c r="G24" s="66" t="n"/>
+      <c r="H24" s="66" t="n"/>
+      <c r="I24" s="66" t="n"/>
+      <c r="J24" s="66" t="n"/>
+      <c r="K24" s="66" t="n"/>
+      <c r="L24" s="73" t="n"/>
+      <c r="M24" s="48" t="n"/>
+      <c r="N24" s="74" t="n"/>
+      <c r="O24" s="75" t="n"/>
+      <c r="P24" s="68" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="23">
+      <c r="A25" s="64" t="inlineStr">
+        <is>
+          <t>N558899</t>
+        </is>
+      </c>
+      <c r="B25" s="64" t="inlineStr">
+        <is>
+          <t>Verlinden</t>
+        </is>
+      </c>
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>Mehdi</t>
+        </is>
+      </c>
+      <c r="D25" s="72" t="n"/>
+      <c r="E25" s="66" t="n"/>
+      <c r="F25" s="66" t="n"/>
+      <c r="G25" s="66" t="n"/>
+      <c r="H25" s="66" t="n"/>
+      <c r="I25" s="66" t="n"/>
+      <c r="J25" s="66" t="n"/>
+      <c r="K25" s="66" t="n"/>
+      <c r="L25" s="73" t="n"/>
+      <c r="M25" s="48" t="n"/>
+      <c r="N25" s="74" t="n"/>
+      <c r="O25" s="75" t="n"/>
+      <c r="P25" s="68" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="23">
+      <c r="A26" s="76" t="inlineStr">
+        <is>
+          <t>P838471</t>
+        </is>
+      </c>
+      <c r="B26" s="76" t="inlineStr">
+        <is>
+          <t>Wahbi</t>
+        </is>
+      </c>
+      <c r="C26" s="76" t="inlineStr">
+        <is>
+          <t>Chaimaa</t>
+        </is>
+      </c>
+      <c r="D26" s="72" t="n"/>
+      <c r="E26" s="66" t="n"/>
+      <c r="F26" s="66" t="n"/>
+      <c r="G26" s="66" t="n"/>
+      <c r="H26" s="66" t="n"/>
+      <c r="I26" s="66" t="n"/>
+      <c r="J26" s="66" t="n"/>
+      <c r="K26" s="66" t="n"/>
+      <c r="L26" s="73" t="n"/>
+      <c r="M26" s="48" t="n"/>
+      <c r="N26" s="74" t="n"/>
+      <c r="O26" s="75" t="n"/>
+      <c r="P26" s="68" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="23">
+      <c r="A27" s="64" t="inlineStr">
+        <is>
+          <t>N180005</t>
+        </is>
+      </c>
+      <c r="B27" s="64" t="inlineStr">
+        <is>
+          <t>Xalil</t>
+        </is>
+      </c>
+      <c r="C27" s="64" t="inlineStr">
+        <is>
+          <t>Driss</t>
+        </is>
+      </c>
+      <c r="D27" s="72" t="n"/>
+      <c r="E27" s="66" t="n"/>
+      <c r="F27" s="66" t="n"/>
+      <c r="G27" s="66" t="n"/>
+      <c r="H27" s="66" t="n"/>
+      <c r="I27" s="66" t="n"/>
+      <c r="J27" s="66" t="n"/>
+      <c r="K27" s="66" t="n"/>
+      <c r="L27" s="73" t="n"/>
+      <c r="M27" s="48" t="n"/>
+      <c r="N27" s="74" t="n"/>
+      <c r="O27" s="75" t="n"/>
+      <c r="P27" s="68" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="23">
+      <c r="A28" s="76" t="inlineStr">
+        <is>
+          <t>F980265</t>
+        </is>
+      </c>
+      <c r="B28" s="76" t="inlineStr">
+        <is>
+          <t>Yahi</t>
+        </is>
+      </c>
+      <c r="C28" s="76" t="inlineStr">
+        <is>
+          <t>Loubna</t>
+        </is>
+      </c>
+      <c r="D28" s="72" t="n"/>
+      <c r="E28" s="66" t="n"/>
+      <c r="F28" s="66" t="n"/>
+      <c r="G28" s="66" t="n"/>
+      <c r="H28" s="66" t="n"/>
+      <c r="I28" s="66" t="n"/>
+      <c r="J28" s="66" t="n"/>
+      <c r="K28" s="66" t="n"/>
+      <c r="L28" s="73" t="n"/>
+      <c r="M28" s="48" t="n"/>
+      <c r="N28" s="74" t="n"/>
+      <c r="O28" s="75" t="n"/>
+      <c r="P28" s="68" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="23">
+      <c r="A29" s="64" t="inlineStr">
+        <is>
+          <t>R879232</t>
+        </is>
+      </c>
+      <c r="B29" s="64" t="inlineStr">
+        <is>
+          <t>Zahraoui</t>
+        </is>
+      </c>
+      <c r="C29" s="64" t="inlineStr">
+        <is>
+          <t>Saad</t>
+        </is>
+      </c>
+      <c r="D29" s="72" t="n"/>
+      <c r="E29" s="66" t="n"/>
+      <c r="F29" s="66" t="n"/>
+      <c r="G29" s="66" t="n"/>
+      <c r="H29" s="66" t="n"/>
+      <c r="I29" s="66" t="n"/>
+      <c r="J29" s="66" t="n"/>
+      <c r="K29" s="66" t="n"/>
+      <c r="L29" s="73" t="n"/>
+      <c r="M29" s="48" t="n"/>
+      <c r="N29" s="74" t="n"/>
+      <c r="O29" s="75" t="n"/>
+      <c r="P29" s="68" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="23">
+      <c r="A30" s="76" t="inlineStr">
+        <is>
+          <t>T991021</t>
+        </is>
+      </c>
+      <c r="B30" s="76" t="inlineStr">
+        <is>
+          <t>Abbadi</t>
+        </is>
+      </c>
+      <c r="C30" s="76" t="inlineStr">
+        <is>
+          <t>Basma</t>
+        </is>
+      </c>
+      <c r="D30" s="72" t="n"/>
+      <c r="E30" s="66" t="n"/>
+      <c r="F30" s="66" t="n"/>
+      <c r="G30" s="66" t="n"/>
+      <c r="H30" s="66" t="n"/>
+      <c r="I30" s="66" t="n"/>
+      <c r="J30" s="66" t="n"/>
+      <c r="K30" s="66" t="n"/>
+      <c r="L30" s="73" t="n"/>
+      <c r="M30" s="48" t="n"/>
+      <c r="N30" s="74" t="n"/>
+      <c r="O30" s="75" t="n"/>
+      <c r="P30" s="68" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="23">
+      <c r="A31" s="64" t="inlineStr">
+        <is>
+          <t>F199535</t>
+        </is>
+      </c>
+      <c r="B31" s="64" t="inlineStr">
+        <is>
+          <t>Bakkali</t>
+        </is>
+      </c>
+      <c r="C31" s="64" t="inlineStr">
+        <is>
+          <t>Ayoub</t>
+        </is>
+      </c>
+      <c r="D31" s="72" t="n"/>
+      <c r="E31" s="66" t="n"/>
+      <c r="F31" s="66" t="n"/>
+      <c r="G31" s="66" t="n"/>
+      <c r="H31" s="66" t="n"/>
+      <c r="I31" s="66" t="n"/>
+      <c r="J31" s="66" t="n"/>
+      <c r="K31" s="66" t="n"/>
+      <c r="L31" s="73" t="n"/>
+      <c r="M31" s="48" t="n"/>
+      <c r="N31" s="74" t="n"/>
+      <c r="O31" s="75" t="n"/>
+      <c r="P31" s="68" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="23">
+      <c r="A32" s="76" t="inlineStr">
+        <is>
+          <t>P583643</t>
+        </is>
+      </c>
+      <c r="B32" s="76" t="inlineStr">
+        <is>
+          <t>Chakir</t>
+        </is>
+      </c>
+      <c r="C32" s="76" t="inlineStr">
+        <is>
+          <t>Sanae</t>
+        </is>
+      </c>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="66" t="n"/>
+      <c r="F32" s="66" t="n"/>
+      <c r="G32" s="66" t="n"/>
+      <c r="H32" s="66" t="n"/>
+      <c r="I32" s="66" t="n"/>
+      <c r="J32" s="66" t="n"/>
+      <c r="K32" s="66" t="n"/>
+      <c r="L32" s="73" t="n"/>
+      <c r="M32" s="48" t="n"/>
+      <c r="N32" s="74" t="n"/>
+      <c r="O32" s="75" t="n"/>
+      <c r="P32" s="68" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="23">
+      <c r="A33" s="64" t="inlineStr">
+        <is>
+          <t>F919533</t>
+        </is>
+      </c>
+      <c r="B33" s="64" t="inlineStr">
+        <is>
+          <t>Darouich</t>
+        </is>
+      </c>
+      <c r="C33" s="64" t="inlineStr">
+        <is>
+          <t>Khalid</t>
+        </is>
+      </c>
+      <c r="D33" s="72" t="n"/>
+      <c r="E33" s="66" t="n"/>
+      <c r="F33" s="66" t="n"/>
+      <c r="G33" s="66" t="n"/>
+      <c r="H33" s="66" t="n"/>
+      <c r="I33" s="66" t="n"/>
+      <c r="J33" s="66" t="n"/>
+      <c r="K33" s="66" t="n"/>
+      <c r="L33" s="73" t="n"/>
+      <c r="M33" s="48" t="n"/>
+      <c r="N33" s="74" t="n"/>
+      <c r="O33" s="75" t="n"/>
+      <c r="P33" s="68" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="23">
+      <c r="A34" s="76" t="inlineStr">
+        <is>
+          <t>N211648</t>
+        </is>
+      </c>
+      <c r="B34" s="76" t="inlineStr">
+        <is>
+          <t>Essalhi</t>
+        </is>
+      </c>
+      <c r="C34" s="76" t="inlineStr">
+        <is>
+          <t>Latifa</t>
+        </is>
+      </c>
+      <c r="D34" s="72" t="n"/>
+      <c r="E34" s="66" t="n"/>
+      <c r="F34" s="66" t="n"/>
+      <c r="G34" s="66" t="n"/>
+      <c r="H34" s="66" t="n"/>
+      <c r="I34" s="66" t="n"/>
+      <c r="J34" s="66" t="n"/>
+      <c r="K34" s="66" t="n"/>
+      <c r="L34" s="73" t="n"/>
+      <c r="M34" s="48" t="n"/>
+      <c r="N34" s="74" t="n"/>
+      <c r="O34" s="75" t="n"/>
+      <c r="P34" s="68" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="23">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>B566362</t>
+        </is>
+      </c>
+      <c r="B35" s="64" t="inlineStr">
+        <is>
+          <t>Figuigui</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>Amine</t>
+        </is>
+      </c>
+      <c r="D35" s="72" t="n"/>
+      <c r="E35" s="66" t="n"/>
+      <c r="F35" s="66" t="n"/>
+      <c r="G35" s="66" t="n"/>
+      <c r="H35" s="66" t="n"/>
+      <c r="I35" s="66" t="n"/>
+      <c r="J35" s="66" t="n"/>
+      <c r="K35" s="66" t="n"/>
+      <c r="L35" s="73" t="n"/>
+      <c r="M35" s="48" t="n"/>
+      <c r="N35" s="74" t="n"/>
+      <c r="O35" s="75" t="n"/>
+      <c r="P35" s="68" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="D2:M2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Purge complete tolerance + Nouveau systeme diagnostic strict (S5/PFE/NV)
- Suppression totale de la logique de tolerance, bonus et passage_tolerant
- Suppression des statuts ORANGE et ORANGE_JURY (ne reste que VERT/JAUNE/ROUGE)
- Renommage VIGILANCE -> RISQUE MODERE dans toute l'application
- Nouvelle classification basee sur 3 criteres: Note S5, Note PFE, Modules NV
  VERT: S5>=12 ET PFE>=12 ET NV<=3
  JAUNE: S5>=11 ET PFE>=12 ET NV<=3
  ROUGE: sinon (avec detail des raisons)
- Compatibilite Diagnostic/Prediction 3A: pas de diagnostic pour etudiants valides
- PFE force a la reussite (pas de rattrapage pour le PFE)
- Dataset mis a jour: notes PFA > 12 pour tous les etudiants
- Fond blanc pour l'interface + texte sombre
- Nettoyage des scripts temporaires et fichiers obsoletes
- 6/6 tests de coherence passes
</commit_message>
<xml_diff>
--- a/data/raw/ccn_cybersec.xlsx
+++ b/data/raw/ccn_cybersec.xlsx
@@ -509,7 +509,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -737,6 +737,8 @@
     <xf numFmtId="0" fontId="18" fillId="39" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2764,68 +2766,68 @@
         <v>17</v>
       </c>
       <c r="E22" s="41" t="n">
-        <v>12.46</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="F22" s="41" t="n">
-        <v>14.67</v>
+        <v>12.32</v>
       </c>
       <c r="G22" s="41" t="n">
-        <v>18.31</v>
+        <v>14.58</v>
       </c>
       <c r="H22" s="41" t="n">
-        <v>15.09</v>
+        <v>11.62</v>
       </c>
       <c r="I22" s="41" t="n">
-        <v>14.19</v>
+        <v>9.67</v>
       </c>
       <c r="J22" s="40" t="n">
-        <v>11.04</v>
+        <v>7.52</v>
       </c>
       <c r="K22" s="40" t="n">
-        <v>10.48</v>
+        <v>6.93</v>
       </c>
       <c r="M22" s="48" t="n">
-        <v>14.1</v>
+        <v>10.24</v>
       </c>
       <c r="N22" s="39" t="n">
         <v>16</v>
       </c>
       <c r="O22" s="41" t="n">
-        <v>12.63</v>
+        <v>10.4</v>
       </c>
       <c r="P22" s="41" t="n">
-        <v>13.08</v>
+        <v>10.07</v>
       </c>
       <c r="Q22" s="41" t="n">
-        <v>13.56</v>
+        <v>10.73</v>
       </c>
       <c r="R22" s="41" t="n">
-        <v>18.49</v>
+        <v>12.09</v>
       </c>
       <c r="S22" s="41" t="n">
-        <v>16.12</v>
+        <v>13.6</v>
       </c>
       <c r="T22" s="40" t="n">
-        <v>8.220000000000001</v>
+        <v>6.71</v>
       </c>
       <c r="U22" s="41" t="n">
-        <v>14.83</v>
+        <v>10.27</v>
       </c>
       <c r="V22" s="41" t="n">
-        <v>13.53</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="W22" s="48" t="n">
-        <v>13.87</v>
+        <v>10.4</v>
       </c>
       <c r="X22" s="49" t="n">
-        <v>13.98</v>
+        <v>10.32</v>
       </c>
       <c r="Y22" s="50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Z22" s="51" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -3699,68 +3701,68 @@
         <v>16</v>
       </c>
       <c r="E33" s="41" t="n">
-        <v>13.08</v>
+        <v>8.98</v>
       </c>
       <c r="F33" s="41" t="n">
-        <v>17.19</v>
+        <v>12.22</v>
       </c>
       <c r="G33" s="40" t="n">
-        <v>10.89</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="H33" s="40" t="n">
-        <v>10.15</v>
+        <v>7.47</v>
       </c>
       <c r="I33" s="41" t="n">
-        <v>13.88</v>
+        <v>9.83</v>
       </c>
       <c r="J33" s="41" t="n">
-        <v>19.2</v>
+        <v>14.83</v>
       </c>
       <c r="K33" s="41" t="n">
-        <v>12.03</v>
+        <v>8.16</v>
       </c>
       <c r="M33" s="48" t="n">
-        <v>13.64</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="N33" s="39" t="n">
         <v>8</v>
       </c>
       <c r="O33" s="40" t="n">
-        <v>11.59</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="P33" s="41" t="n">
-        <v>15.03</v>
+        <v>10.87</v>
       </c>
       <c r="Q33" s="41" t="n">
-        <v>14.41</v>
+        <v>10.68</v>
       </c>
       <c r="R33" s="41" t="n">
-        <v>14.85</v>
+        <v>11.98</v>
       </c>
       <c r="S33" s="41" t="n">
-        <v>18.18</v>
+        <v>12.54</v>
       </c>
       <c r="T33" s="41" t="n">
-        <v>14.66</v>
+        <v>11.04</v>
       </c>
       <c r="U33" s="41" t="n">
-        <v>19.1</v>
+        <v>14.68</v>
       </c>
       <c r="V33" s="41" t="n">
-        <v>12.51</v>
+        <v>8.25</v>
       </c>
       <c r="W33" s="48" t="n">
-        <v>14.74</v>
+        <v>11.03</v>
       </c>
       <c r="X33" s="49" t="n">
-        <v>14.19</v>
+        <v>10.5</v>
       </c>
       <c r="Y33" s="50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Z33" s="51" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -4124,68 +4126,68 @@
         <v>5</v>
       </c>
       <c r="E38" s="41" t="n">
-        <v>12.52</v>
+        <v>9.66</v>
       </c>
       <c r="F38" s="41" t="n">
-        <v>13.89</v>
+        <v>9.5</v>
       </c>
       <c r="G38" s="41" t="n">
-        <v>18.59</v>
+        <v>12.33</v>
       </c>
       <c r="H38" s="41" t="n">
-        <v>16.47</v>
+        <v>13.83</v>
       </c>
       <c r="I38" s="41" t="n">
-        <v>17.91</v>
+        <v>15.1</v>
       </c>
       <c r="J38" s="41" t="n">
-        <v>14.57</v>
+        <v>11.83</v>
       </c>
       <c r="K38" s="41" t="n">
-        <v>14.08</v>
+        <v>10.01</v>
       </c>
       <c r="M38" s="48" t="n">
-        <v>15.46</v>
+        <v>11.75</v>
       </c>
       <c r="N38" s="39" t="n">
         <v>18</v>
       </c>
       <c r="O38" s="41" t="n">
-        <v>18.63</v>
+        <v>12.47</v>
       </c>
       <c r="P38" s="40" t="n">
-        <v>8.65</v>
+        <v>6.81</v>
       </c>
       <c r="Q38" s="41" t="n">
-        <v>14.27</v>
+        <v>10.53</v>
       </c>
       <c r="R38" s="41" t="n">
-        <v>15.48</v>
+        <v>10.44</v>
       </c>
       <c r="S38" s="41" t="n">
-        <v>16.26</v>
+        <v>12.18</v>
       </c>
       <c r="T38" s="40" t="n">
-        <v>11.96</v>
+        <v>7.86</v>
       </c>
       <c r="U38" s="40" t="n">
-        <v>11.52</v>
+        <v>9.58</v>
       </c>
       <c r="V38" s="41" t="n">
-        <v>16.39</v>
+        <v>11.5</v>
       </c>
       <c r="W38" s="48" t="n">
-        <v>14.33</v>
+        <v>10.17</v>
       </c>
       <c r="X38" s="49" t="n">
-        <v>14.89</v>
+        <v>10.96</v>
       </c>
       <c r="Y38" s="50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Z38" s="51" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="22" min="1" max="1"/>
@@ -7485,7 +7487,7 @@
         <v>11.04</v>
       </c>
       <c r="Y38" s="50" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Z38" s="52" t="inlineStr">
         <is>
@@ -7578,7 +7580,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="N2:W2"/>
@@ -7626,6 +7627,21 @@
           <t>DÉPARTEMENT CCN CYBERSÉCURITÉ — TROISIÈME ANNÉE</t>
         </is>
       </c>
+      <c r="B1" s="77" t="n"/>
+      <c r="C1" s="77" t="n"/>
+      <c r="D1" s="77" t="n"/>
+      <c r="E1" s="77" t="n"/>
+      <c r="F1" s="77" t="n"/>
+      <c r="G1" s="77" t="n"/>
+      <c r="H1" s="77" t="n"/>
+      <c r="I1" s="77" t="n"/>
+      <c r="J1" s="77" t="n"/>
+      <c r="K1" s="77" t="n"/>
+      <c r="L1" s="77" t="n"/>
+      <c r="M1" s="77" t="n"/>
+      <c r="N1" s="77" t="n"/>
+      <c r="O1" s="77" t="n"/>
+      <c r="P1" s="78" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1" s="23">
       <c r="A2" s="54" t="inlineStr">
@@ -7633,11 +7649,22 @@
           <t>Informations Générales</t>
         </is>
       </c>
+      <c r="B2" s="77" t="n"/>
+      <c r="C2" s="78" t="n"/>
       <c r="D2" s="54" t="inlineStr">
         <is>
           <t>SEMESTRE 5</t>
         </is>
       </c>
+      <c r="E2" s="77" t="n"/>
+      <c r="F2" s="77" t="n"/>
+      <c r="G2" s="77" t="n"/>
+      <c r="H2" s="77" t="n"/>
+      <c r="I2" s="77" t="n"/>
+      <c r="J2" s="77" t="n"/>
+      <c r="K2" s="77" t="n"/>
+      <c r="L2" s="77" t="n"/>
+      <c r="M2" s="78" t="n"/>
       <c r="N2" s="54" t="inlineStr">
         <is>
           <t>SEMESTRE 6</t>
@@ -7648,6 +7675,8 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="23">
       <c r="A3" s="55" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="78" t="n"/>
       <c r="D3" s="56" t="n"/>
       <c r="E3" s="56" t="inlineStr">
         <is>

</xml_diff>